<commit_message>
Reconcile v5.7.1 RC6 report evidence
</commit_message>
<xml_diff>
--- a/audits/evidence/v571_rc6_candidate/report/01_biological_results/Biological_Comparison_Data.xlsx
+++ b/audits/evidence/v571_rc6_candidate/report/01_biological_results/Biological_Comparison_Data.xlsx
@@ -277,67 +277,67 @@
     <t>pdf_token</t>
   </si>
   <si>
-    <t>8.952</t>
-  </si>
-  <si>
-    <t>1.692</t>
-  </si>
-  <si>
-    <t>5.9315</t>
-  </si>
-  <si>
-    <t>9.29183</t>
-  </si>
-  <si>
-    <t>1.17993</t>
-  </si>
-  <si>
-    <t>1.43757</t>
-  </si>
-  <si>
-    <t>14.7234</t>
-  </si>
-  <si>
-    <t>10.52</t>
-  </si>
-  <si>
-    <t>1.558</t>
-  </si>
-  <si>
-    <t>7.39855</t>
-  </si>
-  <si>
-    <t>10.9169</t>
-  </si>
-  <si>
-    <t>1.2195</t>
-  </si>
-  <si>
-    <t>1.41056</t>
-  </si>
-  <si>
-    <t>17.1525</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_2d_length_um REF=8.952 COMP=10.52</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_body_width_um REF=1.692 COMP=1.558</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_length_body_width_ratio REF=5.9315 COMP=7.39855</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_projection_z_extent_um REF=9.29183 COMP=10.9169</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_3d_tortuosity REF=1.17993 COMP=1.2195</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_observed_slab_effective_thickness_um REF=1.43757 COMP=1.41056</t>
-  </si>
-  <si>
-    <t>SOURCE_VALUE median_observed_slice_mask_volume_um3 REF=14.7234 COMP=17.1525</t>
+    <t>8.536</t>
+  </si>
+  <si>
+    <t>1.6921</t>
+  </si>
+  <si>
+    <t>5.71658</t>
+  </si>
+  <si>
+    <t>8.91293</t>
+  </si>
+  <si>
+    <t>1.12374</t>
+  </si>
+  <si>
+    <t>1.28161</t>
+  </si>
+  <si>
+    <t>11.7489</t>
+  </si>
+  <si>
+    <t>9.92</t>
+  </si>
+  <si>
+    <t>1.5523</t>
+  </si>
+  <si>
+    <t>7.04507</t>
+  </si>
+  <si>
+    <t>10.197</t>
+  </si>
+  <si>
+    <t>1.13236</t>
+  </si>
+  <si>
+    <t>1.26257</t>
+  </si>
+  <si>
+    <t>13.0379</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_2d_length_um REF=8.536 COMP=9.92</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_body_width_um REF=1.6921 COMP=1.5523</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_length_body_width_ratio REF=5.71658 COMP=7.04507</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_projection_z_extent_um REF=8.91293 COMP=10.197</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_3d_tortuosity REF=1.12374 COMP=1.13236</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_observed_slab_effective_thickness_um REF=1.28161 COMP=1.26257</t>
+  </si>
+  <si>
+    <t>SOURCE_VALUE median_observed_slice_mask_volume_um3 REF=11.7489 COMP=13.0379</t>
   </si>
   <si>
     <t>biological_question</t>
@@ -886,25 +886,25 @@
         <v>24</v>
       </c>
       <c r="D2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="E2">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="F2">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="G2">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="H2">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="I2">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="J2">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -918,25 +918,25 @@
         <v>24</v>
       </c>
       <c r="D3">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="E3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="F3">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="G3">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="H3">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="I3">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="J3">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
     </row>
   </sheetData>
@@ -998,25 +998,25 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="D2">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="E2">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="F2">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="G2">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="H2">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="I2">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1027,25 +1027,25 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="D3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="E3">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="F3">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="G3">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="H3">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="I3">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
     </row>
   </sheetData>
@@ -1224,34 +1224,34 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="L2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="O2">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="P2">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="Q2">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="R2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="S2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="T2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="U2">
-        <v>1.568</v>
+        <v>1.384</v>
       </c>
       <c r="V2">
-        <v>17.51563896336014</v>
+        <v>16.21368322399251</v>
       </c>
     </row>
     <row r="3" spans="1:34">
@@ -1286,34 +1286,34 @@
         <v>1</v>
       </c>
       <c r="K3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="L3">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="O3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="P3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="Q3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="R3">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="S3">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="T3">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="U3">
-        <v>-0.1339999999999999</v>
+        <v>-0.1397999999999999</v>
       </c>
       <c r="V3">
-        <v>-7.919621749408978</v>
+        <v>-8.26192305419301</v>
       </c>
     </row>
     <row r="4" spans="1:34">
@@ -1348,34 +1348,34 @@
         <v>1</v>
       </c>
       <c r="K4">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="L4">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="O4">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="P4">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="Q4">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="R4">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="S4">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="T4">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="U4">
-        <v>1.467044265106946</v>
+        <v>1.328489811471443</v>
       </c>
       <c r="V4">
-        <v>24.73308789101713</v>
+        <v>23.2392294594024</v>
       </c>
     </row>
     <row r="5" spans="1:34">
@@ -1410,34 +1410,34 @@
         <v>1</v>
       </c>
       <c r="K5">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="L5">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="O5">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="P5">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="Q5">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="R5">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="S5">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="T5">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="U5">
-        <v>1.625051976393541</v>
+        <v>1.284054884741034</v>
       </c>
       <c r="V5">
-        <v>17.48903866264752</v>
+        <v>14.40665395685874</v>
       </c>
     </row>
     <row r="6" spans="1:34">
@@ -1472,34 +1472,34 @@
         <v>1</v>
       </c>
       <c r="K6">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="L6">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="O6">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="P6">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="Q6">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="R6">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="S6">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="T6">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="U6">
-        <v>0.03957384942914643</v>
+        <v>0.008622635148719082</v>
       </c>
       <c r="V6">
-        <v>3.353918119731329</v>
+        <v>0.7673162873989298</v>
       </c>
     </row>
     <row r="7" spans="1:34">
@@ -1534,34 +1534,34 @@
         <v>1</v>
       </c>
       <c r="K7">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="L7">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="O7">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="P7">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="Q7">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="R7">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="S7">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="T7">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="U7">
-        <v>-0.02701317754520138</v>
+        <v>-0.01904232634781033</v>
       </c>
       <c r="V7">
-        <v>-1.87908014175313</v>
+        <v>-1.485814965141742</v>
       </c>
     </row>
     <row r="8" spans="1:34">
@@ -1596,34 +1596,34 @@
         <v>1</v>
       </c>
       <c r="K8">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
       <c r="L8">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
       <c r="O8">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
       <c r="P8">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
       <c r="Q8">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
       <c r="R8">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
       <c r="S8">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
       <c r="T8">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
       <c r="U8">
-        <v>2.42910734037072</v>
+        <v>1.288914098972214</v>
       </c>
       <c r="V8">
-        <v>16.49831649831639</v>
+        <v>10.97046413502098</v>
       </c>
     </row>
   </sheetData>
@@ -1690,10 +1690,10 @@
         <v>8</v>
       </c>
       <c r="E2">
-        <v>8.952</v>
+        <v>8.536</v>
       </c>
       <c r="F2">
-        <v>10.52</v>
+        <v>9.92</v>
       </c>
       <c r="G2" t="s">
         <v>82</v>
@@ -1719,10 +1719,10 @@
         <v>8</v>
       </c>
       <c r="E3">
-        <v>1.692</v>
+        <v>1.6921</v>
       </c>
       <c r="F3">
-        <v>1.558</v>
+        <v>1.5523</v>
       </c>
       <c r="G3" t="s">
         <v>83</v>
@@ -1748,10 +1748,10 @@
         <v>8</v>
       </c>
       <c r="E4">
-        <v>5.931504677342636</v>
+        <v>5.716582874626884</v>
       </c>
       <c r="F4">
-        <v>7.398548942449581</v>
+        <v>7.045072686098327</v>
       </c>
       <c r="G4" t="s">
         <v>84</v>
@@ -1777,10 +1777,10 @@
         <v>8</v>
       </c>
       <c r="E5">
-        <v>9.291831344991367</v>
+        <v>8.912929321313497</v>
       </c>
       <c r="F5">
-        <v>10.91688332138491</v>
+        <v>10.19698420605453</v>
       </c>
       <c r="G5" t="s">
         <v>85</v>
@@ -1806,10 +1806,10 @@
         <v>8</v>
       </c>
       <c r="E6">
-        <v>1.179928907516578</v>
+        <v>1.123739361502195</v>
       </c>
       <c r="F6">
-        <v>1.219502756945725</v>
+        <v>1.132361996650914</v>
       </c>
       <c r="G6" t="s">
         <v>86</v>
@@ -1835,10 +1835,10 @@
         <v>8</v>
       </c>
       <c r="E7">
-        <v>1.43757453154706</v>
+        <v>1.281608194462744</v>
       </c>
       <c r="F7">
-        <v>1.410561354001858</v>
+        <v>1.262565868114934</v>
       </c>
       <c r="G7" t="s">
         <v>87</v>
@@ -1864,10 +1864,10 @@
         <v>8</v>
       </c>
       <c r="E8">
-        <v>14.72336489979814</v>
+        <v>11.74894774832377</v>
       </c>
       <c r="F8">
-        <v>17.15247224016886</v>
+        <v>13.03786184729598</v>
       </c>
       <c r="G8" t="s">
         <v>88</v>

</xml_diff>